<commit_message>
Publish Augsburg_2018_WC, Augsburg_2023_WC, Bratislava_2021_WCH, Krakow_2018_WC
</commit_message>
<xml_diff>
--- a/events/Augsburg_2018_WC/Augsburg_2018_WC_start.xlsx
+++ b/events/Augsburg_2018_WC/Augsburg_2018_WC_start.xlsx
@@ -32540,6 +32540,11 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
+      <c r="X547" t="inlineStr">
+        <is>
+          <t>51837</t>
+        </is>
+      </c>
       <c r="Y547" t="inlineStr">
         <is>
           <t>35135</t>
@@ -32739,6 +32744,11 @@
           <t>POCHWALA Marcin</t>
         </is>
       </c>
+      <c r="X550" t="inlineStr">
+        <is>
+          <t>61261</t>
+        </is>
+      </c>
       <c r="Y550" t="inlineStr">
         <is>
           <t>35079</t>
@@ -32938,6 +32948,11 @@
           <t>JANE Jakub</t>
         </is>
       </c>
+      <c r="X553" t="inlineStr">
+        <is>
+          <t>42016</t>
+        </is>
+      </c>
       <c r="Y553" t="inlineStr">
         <is>
           <t>35061</t>
@@ -33401,6 +33416,11 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
+      <c r="X559" t="inlineStr">
+        <is>
+          <t>51837</t>
+        </is>
+      </c>
       <c r="Y559" t="inlineStr">
         <is>
           <t>35135</t>
@@ -33552,6 +33572,11 @@
           <t>POCHWALA Marcin</t>
         </is>
       </c>
+      <c r="X561" t="inlineStr">
+        <is>
+          <t>61261</t>
+        </is>
+      </c>
       <c r="Y561" t="inlineStr">
         <is>
           <t>35079</t>
@@ -33701,6 +33726,11 @@
       <c r="S563" t="inlineStr">
         <is>
           <t>JANE Jakub</t>
+        </is>
+      </c>
+      <c r="X563" t="inlineStr">
+        <is>
+          <t>42016</t>
         </is>
       </c>
       <c r="Y563" t="inlineStr">

</xml_diff>